<commit_message>
remove resolution from SDRF
</commit_message>
<xml_diff>
--- a/docs/metabobank/metadata_excel/MetaboBank_GCGC-MS_metadata.xlsx
+++ b/docs/metabobank/metadata_excel/MetaboBank_GCGC-MS_metadata.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89D7203-4E65-4D4B-9EDD-60875134BE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F7C5E8-C40A-4B54-9071-62CB7CB83FCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="12" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="195">
   <si>
     <t>Study Title</t>
   </si>
@@ -616,10 +616,6 @@
   </si>
   <si>
     <t>normalization testing design</t>
-  </si>
-  <si>
-    <t>Parameter Value[Resolution 1]</t>
-    <phoneticPr fontId="1"/>
   </si>
   <si>
     <r>
@@ -634,10 +630,6 @@
       </rPr>
       <t>]</t>
     </r>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Parameter Value[Resolution 2]</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -1249,7 +1241,7 @@
         <v>146</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -1283,18 +1275,18 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -1546,7 +1538,7 @@
         <v>125</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>173</v>
@@ -1715,7 +1707,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AN105"/>
+  <dimension ref="A1:AL105"/>
   <sheetFormatPr defaultColWidth="24.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
@@ -1731,46 +1723,46 @@
     <col min="11" max="11" width="40.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="35.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="33.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="33.6640625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="35" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="20" width="35" style="1" customWidth="1"/>
-    <col min="21" max="21" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="33.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="36.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="32.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="15.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="37.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="26.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="29.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="45" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="28.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="16384" width="24.88671875" style="1"/>
+    <col min="14" max="14" width="33.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="35" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="35" style="1" customWidth="1"/>
+    <col min="19" max="19" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="33.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="36.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="34.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="32.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="37.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="26.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="29.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="45" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="28.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="16384" width="24.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
     </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>28</v>
       </c>
@@ -1814,85 +1806,79 @@
         <v>188</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>189</v>
+        <v>37</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>37</v>
+        <v>171</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>190</v>
+        <v>38</v>
       </c>
       <c r="T4" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="U4" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="U4" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="V4" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="W4" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="W4" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="X4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z4" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA4" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD4" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="AE4" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="X4" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y4" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="Z4" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="AA4" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB4" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="AC4" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="AD4" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="AE4" s="8" t="s">
-        <v>47</v>
-      </c>
       <c r="AF4" s="8" t="s">
-        <v>131</v>
+        <v>48</v>
       </c>
       <c r="AG4" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="AH4" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="AH4" s="8" t="s">
-        <v>48</v>
-      </c>
       <c r="AI4" s="8" t="s">
-        <v>130</v>
+        <v>49</v>
       </c>
       <c r="AJ4" s="8" t="s">
-        <v>30</v>
+        <v>132</v>
       </c>
       <c r="AK4" s="8" t="s">
-        <v>49</v>
+        <v>133</v>
       </c>
       <c r="AL4" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="AM4" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="AN4" s="8" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
       <c r="B5" s="11"/>
       <c r="C5" s="11" t="s">
@@ -1919,11 +1905,11 @@
       <c r="R5" s="11"/>
       <c r="S5" s="11"/>
       <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
+      <c r="U5" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="V5" s="11"/>
-      <c r="W5" s="11" t="s">
-        <v>54</v>
-      </c>
+      <c r="W5" s="11"/>
       <c r="X5" s="11"/>
       <c r="Y5" s="11"/>
       <c r="Z5" s="11"/>
@@ -1931,22 +1917,20 @@
       <c r="AB5" s="11"/>
       <c r="AC5" s="11"/>
       <c r="AD5" s="11"/>
-      <c r="AE5" s="11"/>
+      <c r="AE5" s="11" t="s">
+        <v>55</v>
+      </c>
       <c r="AF5" s="11"/>
-      <c r="AG5" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH5" s="11"/>
+      <c r="AG5" s="11"/>
+      <c r="AH5" s="11" t="s">
+        <v>56</v>
+      </c>
       <c r="AI5" s="11"/>
-      <c r="AJ5" s="11" t="s">
-        <v>56</v>
-      </c>
+      <c r="AJ5" s="11"/>
       <c r="AK5" s="11"/>
       <c r="AL5" s="11"/>
-      <c r="AM5" s="11"/>
-      <c r="AN5" s="11"/>
-    </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11" t="s">
@@ -1973,11 +1957,11 @@
       <c r="R6" s="11"/>
       <c r="S6" s="11"/>
       <c r="T6" s="11"/>
-      <c r="U6" s="11"/>
+      <c r="U6" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="V6" s="11"/>
-      <c r="W6" s="11" t="s">
-        <v>54</v>
-      </c>
+      <c r="W6" s="11"/>
       <c r="X6" s="11"/>
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
@@ -1985,22 +1969,20 @@
       <c r="AB6" s="11"/>
       <c r="AC6" s="11"/>
       <c r="AD6" s="11"/>
-      <c r="AE6" s="11"/>
+      <c r="AE6" s="11" t="s">
+        <v>55</v>
+      </c>
       <c r="AF6" s="11"/>
-      <c r="AG6" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH6" s="11"/>
+      <c r="AG6" s="11"/>
+      <c r="AH6" s="11" t="s">
+        <v>56</v>
+      </c>
       <c r="AI6" s="11"/>
-      <c r="AJ6" s="11" t="s">
-        <v>56</v>
-      </c>
+      <c r="AJ6" s="11"/>
       <c r="AK6" s="11"/>
       <c r="AL6" s="11"/>
-      <c r="AM6" s="11"/>
-      <c r="AN6" s="11"/>
-    </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11" t="s">
@@ -2027,11 +2009,11 @@
       <c r="R7" s="11"/>
       <c r="S7" s="11"/>
       <c r="T7" s="11"/>
-      <c r="U7" s="11"/>
+      <c r="U7" s="11" t="s">
+        <v>54</v>
+      </c>
       <c r="V7" s="11"/>
-      <c r="W7" s="11" t="s">
-        <v>54</v>
-      </c>
+      <c r="W7" s="11"/>
       <c r="X7" s="11"/>
       <c r="Y7" s="11"/>
       <c r="Z7" s="11"/>
@@ -2039,22 +2021,20 @@
       <c r="AB7" s="11"/>
       <c r="AC7" s="11"/>
       <c r="AD7" s="11"/>
-      <c r="AE7" s="11"/>
+      <c r="AE7" s="11" t="s">
+        <v>55</v>
+      </c>
       <c r="AF7" s="11"/>
-      <c r="AG7" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="AH7" s="11"/>
+      <c r="AG7" s="11"/>
+      <c r="AH7" s="11" t="s">
+        <v>56</v>
+      </c>
       <c r="AI7" s="11"/>
-      <c r="AJ7" s="11" t="s">
-        <v>56</v>
-      </c>
+      <c r="AJ7" s="11"/>
       <c r="AK7" s="11"/>
       <c r="AL7" s="11"/>
-      <c r="AM7" s="11"/>
-      <c r="AN7" s="11"/>
-    </row>
-    <row r="8" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="12"/>
@@ -2093,10 +2073,8 @@
       <c r="AJ8" s="11"/>
       <c r="AK8" s="11"/>
       <c r="AL8" s="11"/>
-      <c r="AM8" s="11"/>
-      <c r="AN8" s="11"/>
-    </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
       <c r="C9" s="12"/>
@@ -2135,10 +2113,8 @@
       <c r="AJ9" s="11"/>
       <c r="AK9" s="11"/>
       <c r="AL9" s="11"/>
-      <c r="AM9" s="11"/>
-      <c r="AN9" s="11"/>
-    </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
       <c r="B10" s="11"/>
       <c r="C10" s="12"/>
@@ -2177,10 +2153,8 @@
       <c r="AJ10" s="11"/>
       <c r="AK10" s="11"/>
       <c r="AL10" s="11"/>
-      <c r="AM10" s="11"/>
-      <c r="AN10" s="11"/>
-    </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
       <c r="B11" s="11"/>
       <c r="C11" s="12"/>
@@ -2219,10 +2193,8 @@
       <c r="AJ11" s="11"/>
       <c r="AK11" s="11"/>
       <c r="AL11" s="11"/>
-      <c r="AM11" s="11"/>
-      <c r="AN11" s="11"/>
-    </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="12"/>
@@ -2261,10 +2233,8 @@
       <c r="AJ12" s="11"/>
       <c r="AK12" s="11"/>
       <c r="AL12" s="11"/>
-      <c r="AM12" s="11"/>
-      <c r="AN12" s="11"/>
-    </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="12"/>
@@ -2303,10 +2273,8 @@
       <c r="AJ13" s="11"/>
       <c r="AK13" s="11"/>
       <c r="AL13" s="11"/>
-      <c r="AM13" s="11"/>
-      <c r="AN13" s="11"/>
-    </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="12"/>
@@ -2345,10 +2313,8 @@
       <c r="AJ14" s="11"/>
       <c r="AK14" s="11"/>
       <c r="AL14" s="11"/>
-      <c r="AM14" s="11"/>
-      <c r="AN14" s="11"/>
-    </row>
-    <row r="15" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="12"/>
@@ -2387,10 +2353,8 @@
       <c r="AJ15" s="11"/>
       <c r="AK15" s="11"/>
       <c r="AL15" s="11"/>
-      <c r="AM15" s="11"/>
-      <c r="AN15" s="11"/>
-    </row>
-    <row r="16" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="12"/>
@@ -2429,10 +2393,8 @@
       <c r="AJ16" s="11"/>
       <c r="AK16" s="11"/>
       <c r="AL16" s="11"/>
-      <c r="AM16" s="11"/>
-      <c r="AN16" s="11"/>
-    </row>
-    <row r="17" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="12"/>
@@ -2471,10 +2433,8 @@
       <c r="AJ17" s="11"/>
       <c r="AK17" s="11"/>
       <c r="AL17" s="11"/>
-      <c r="AM17" s="11"/>
-      <c r="AN17" s="11"/>
-    </row>
-    <row r="18" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="12"/>
@@ -2513,10 +2473,8 @@
       <c r="AJ18" s="11"/>
       <c r="AK18" s="11"/>
       <c r="AL18" s="11"/>
-      <c r="AM18" s="11"/>
-      <c r="AN18" s="11"/>
-    </row>
-    <row r="19" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="12"/>
@@ -2555,10 +2513,8 @@
       <c r="AJ19" s="11"/>
       <c r="AK19" s="11"/>
       <c r="AL19" s="11"/>
-      <c r="AM19" s="11"/>
-      <c r="AN19" s="11"/>
-    </row>
-    <row r="20" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
       <c r="B20" s="11"/>
       <c r="C20" s="12"/>
@@ -2597,10 +2553,8 @@
       <c r="AJ20" s="11"/>
       <c r="AK20" s="11"/>
       <c r="AL20" s="11"/>
-      <c r="AM20" s="11"/>
-      <c r="AN20" s="11"/>
-    </row>
-    <row r="21" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="B21" s="11"/>
       <c r="C21" s="12"/>
@@ -2639,10 +2593,8 @@
       <c r="AJ21" s="11"/>
       <c r="AK21" s="11"/>
       <c r="AL21" s="11"/>
-      <c r="AM21" s="11"/>
-      <c r="AN21" s="11"/>
-    </row>
-    <row r="22" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
       <c r="B22" s="11"/>
       <c r="C22" s="12"/>
@@ -2681,10 +2633,8 @@
       <c r="AJ22" s="11"/>
       <c r="AK22" s="11"/>
       <c r="AL22" s="11"/>
-      <c r="AM22" s="11"/>
-      <c r="AN22" s="11"/>
-    </row>
-    <row r="23" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A23" s="11"/>
       <c r="B23" s="11"/>
       <c r="C23" s="12"/>
@@ -2723,10 +2673,8 @@
       <c r="AJ23" s="11"/>
       <c r="AK23" s="11"/>
       <c r="AL23" s="11"/>
-      <c r="AM23" s="11"/>
-      <c r="AN23" s="11"/>
-    </row>
-    <row r="24" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A24" s="11"/>
       <c r="B24" s="11"/>
       <c r="C24" s="12"/>
@@ -2765,10 +2713,8 @@
       <c r="AJ24" s="11"/>
       <c r="AK24" s="11"/>
       <c r="AL24" s="11"/>
-      <c r="AM24" s="11"/>
-      <c r="AN24" s="11"/>
-    </row>
-    <row r="25" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="12"/>
@@ -2807,10 +2753,8 @@
       <c r="AJ25" s="11"/>
       <c r="AK25" s="11"/>
       <c r="AL25" s="11"/>
-      <c r="AM25" s="11"/>
-      <c r="AN25" s="11"/>
-    </row>
-    <row r="26" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A26" s="11"/>
       <c r="B26" s="11"/>
       <c r="C26" s="12"/>
@@ -2849,10 +2793,8 @@
       <c r="AJ26" s="11"/>
       <c r="AK26" s="11"/>
       <c r="AL26" s="11"/>
-      <c r="AM26" s="11"/>
-      <c r="AN26" s="11"/>
-    </row>
-    <row r="27" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A27" s="11"/>
       <c r="B27" s="11"/>
       <c r="C27" s="12"/>
@@ -2891,10 +2833,8 @@
       <c r="AJ27" s="11"/>
       <c r="AK27" s="11"/>
       <c r="AL27" s="11"/>
-      <c r="AM27" s="11"/>
-      <c r="AN27" s="11"/>
-    </row>
-    <row r="28" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A28" s="11"/>
       <c r="B28" s="11"/>
       <c r="C28" s="12"/>
@@ -2933,10 +2873,8 @@
       <c r="AJ28" s="11"/>
       <c r="AK28" s="11"/>
       <c r="AL28" s="11"/>
-      <c r="AM28" s="11"/>
-      <c r="AN28" s="11"/>
-    </row>
-    <row r="29" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A29" s="11"/>
       <c r="B29" s="11"/>
       <c r="C29" s="12"/>
@@ -2975,10 +2913,8 @@
       <c r="AJ29" s="11"/>
       <c r="AK29" s="11"/>
       <c r="AL29" s="11"/>
-      <c r="AM29" s="11"/>
-      <c r="AN29" s="11"/>
-    </row>
-    <row r="30" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A30" s="11"/>
       <c r="B30" s="11"/>
       <c r="C30" s="12"/>
@@ -3017,10 +2953,8 @@
       <c r="AJ30" s="11"/>
       <c r="AK30" s="11"/>
       <c r="AL30" s="11"/>
-      <c r="AM30" s="11"/>
-      <c r="AN30" s="11"/>
-    </row>
-    <row r="31" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A31" s="11"/>
       <c r="B31" s="11"/>
       <c r="C31" s="12"/>
@@ -3059,10 +2993,8 @@
       <c r="AJ31" s="11"/>
       <c r="AK31" s="11"/>
       <c r="AL31" s="11"/>
-      <c r="AM31" s="11"/>
-      <c r="AN31" s="11"/>
-    </row>
-    <row r="32" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A32" s="11"/>
       <c r="B32" s="11"/>
       <c r="C32" s="12"/>
@@ -3101,10 +3033,8 @@
       <c r="AJ32" s="11"/>
       <c r="AK32" s="11"/>
       <c r="AL32" s="11"/>
-      <c r="AM32" s="11"/>
-      <c r="AN32" s="11"/>
-    </row>
-    <row r="33" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A33" s="11"/>
       <c r="B33" s="11"/>
       <c r="C33" s="12"/>
@@ -3143,10 +3073,8 @@
       <c r="AJ33" s="11"/>
       <c r="AK33" s="11"/>
       <c r="AL33" s="11"/>
-      <c r="AM33" s="11"/>
-      <c r="AN33" s="11"/>
-    </row>
-    <row r="34" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A34" s="11"/>
       <c r="B34" s="11"/>
       <c r="C34" s="12"/>
@@ -3185,10 +3113,8 @@
       <c r="AJ34" s="11"/>
       <c r="AK34" s="11"/>
       <c r="AL34" s="11"/>
-      <c r="AM34" s="11"/>
-      <c r="AN34" s="11"/>
-    </row>
-    <row r="35" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A35" s="11"/>
       <c r="B35" s="11"/>
       <c r="C35" s="12"/>
@@ -3227,10 +3153,8 @@
       <c r="AJ35" s="11"/>
       <c r="AK35" s="11"/>
       <c r="AL35" s="11"/>
-      <c r="AM35" s="11"/>
-      <c r="AN35" s="11"/>
-    </row>
-    <row r="36" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A36" s="11"/>
       <c r="B36" s="11"/>
       <c r="C36" s="12"/>
@@ -3269,10 +3193,8 @@
       <c r="AJ36" s="11"/>
       <c r="AK36" s="11"/>
       <c r="AL36" s="11"/>
-      <c r="AM36" s="11"/>
-      <c r="AN36" s="11"/>
-    </row>
-    <row r="37" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A37" s="11"/>
       <c r="B37" s="11"/>
       <c r="C37" s="12"/>
@@ -3311,10 +3233,8 @@
       <c r="AJ37" s="11"/>
       <c r="AK37" s="11"/>
       <c r="AL37" s="11"/>
-      <c r="AM37" s="11"/>
-      <c r="AN37" s="11"/>
-    </row>
-    <row r="38" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A38" s="11"/>
       <c r="B38" s="11"/>
       <c r="C38" s="12"/>
@@ -3353,10 +3273,8 @@
       <c r="AJ38" s="11"/>
       <c r="AK38" s="11"/>
       <c r="AL38" s="11"/>
-      <c r="AM38" s="11"/>
-      <c r="AN38" s="11"/>
-    </row>
-    <row r="39" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A39" s="11"/>
       <c r="B39" s="11"/>
       <c r="C39" s="12"/>
@@ -3395,10 +3313,8 @@
       <c r="AJ39" s="11"/>
       <c r="AK39" s="11"/>
       <c r="AL39" s="11"/>
-      <c r="AM39" s="11"/>
-      <c r="AN39" s="11"/>
-    </row>
-    <row r="40" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A40" s="11"/>
       <c r="B40" s="11"/>
       <c r="C40" s="12"/>
@@ -3437,10 +3353,8 @@
       <c r="AJ40" s="11"/>
       <c r="AK40" s="11"/>
       <c r="AL40" s="11"/>
-      <c r="AM40" s="11"/>
-      <c r="AN40" s="11"/>
-    </row>
-    <row r="41" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A41" s="11"/>
       <c r="B41" s="11"/>
       <c r="C41" s="12"/>
@@ -3479,10 +3393,8 @@
       <c r="AJ41" s="11"/>
       <c r="AK41" s="11"/>
       <c r="AL41" s="11"/>
-      <c r="AM41" s="11"/>
-      <c r="AN41" s="11"/>
-    </row>
-    <row r="42" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A42" s="11"/>
       <c r="B42" s="11"/>
       <c r="C42" s="12"/>
@@ -3521,10 +3433,8 @@
       <c r="AJ42" s="11"/>
       <c r="AK42" s="11"/>
       <c r="AL42" s="11"/>
-      <c r="AM42" s="11"/>
-      <c r="AN42" s="11"/>
-    </row>
-    <row r="43" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A43" s="11"/>
       <c r="B43" s="11"/>
       <c r="C43" s="12"/>
@@ -3563,10 +3473,8 @@
       <c r="AJ43" s="11"/>
       <c r="AK43" s="11"/>
       <c r="AL43" s="11"/>
-      <c r="AM43" s="11"/>
-      <c r="AN43" s="11"/>
-    </row>
-    <row r="44" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A44" s="11"/>
       <c r="B44" s="11"/>
       <c r="C44" s="12"/>
@@ -3605,10 +3513,8 @@
       <c r="AJ44" s="11"/>
       <c r="AK44" s="11"/>
       <c r="AL44" s="11"/>
-      <c r="AM44" s="11"/>
-      <c r="AN44" s="11"/>
-    </row>
-    <row r="45" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A45" s="11"/>
       <c r="B45" s="11"/>
       <c r="C45" s="12"/>
@@ -3647,10 +3553,8 @@
       <c r="AJ45" s="11"/>
       <c r="AK45" s="11"/>
       <c r="AL45" s="11"/>
-      <c r="AM45" s="11"/>
-      <c r="AN45" s="11"/>
-    </row>
-    <row r="46" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A46" s="11"/>
       <c r="B46" s="11"/>
       <c r="C46" s="12"/>
@@ -3689,10 +3593,8 @@
       <c r="AJ46" s="11"/>
       <c r="AK46" s="11"/>
       <c r="AL46" s="11"/>
-      <c r="AM46" s="11"/>
-      <c r="AN46" s="11"/>
-    </row>
-    <row r="47" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A47" s="11"/>
       <c r="B47" s="11"/>
       <c r="C47" s="12"/>
@@ -3731,10 +3633,8 @@
       <c r="AJ47" s="11"/>
       <c r="AK47" s="11"/>
       <c r="AL47" s="11"/>
-      <c r="AM47" s="11"/>
-      <c r="AN47" s="11"/>
-    </row>
-    <row r="48" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A48" s="11"/>
       <c r="B48" s="11"/>
       <c r="C48" s="12"/>
@@ -3773,10 +3673,8 @@
       <c r="AJ48" s="11"/>
       <c r="AK48" s="11"/>
       <c r="AL48" s="11"/>
-      <c r="AM48" s="11"/>
-      <c r="AN48" s="11"/>
-    </row>
-    <row r="49" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A49" s="11"/>
       <c r="B49" s="11"/>
       <c r="C49" s="12"/>
@@ -3815,10 +3713,8 @@
       <c r="AJ49" s="11"/>
       <c r="AK49" s="11"/>
       <c r="AL49" s="11"/>
-      <c r="AM49" s="11"/>
-      <c r="AN49" s="11"/>
-    </row>
-    <row r="50" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A50" s="11"/>
       <c r="B50" s="11"/>
       <c r="C50" s="12"/>
@@ -3857,10 +3753,8 @@
       <c r="AJ50" s="11"/>
       <c r="AK50" s="11"/>
       <c r="AL50" s="11"/>
-      <c r="AM50" s="11"/>
-      <c r="AN50" s="11"/>
-    </row>
-    <row r="51" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A51" s="11"/>
       <c r="B51" s="11"/>
       <c r="C51" s="12"/>
@@ -3899,10 +3793,8 @@
       <c r="AJ51" s="11"/>
       <c r="AK51" s="11"/>
       <c r="AL51" s="11"/>
-      <c r="AM51" s="11"/>
-      <c r="AN51" s="11"/>
-    </row>
-    <row r="52" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A52" s="11"/>
       <c r="B52" s="11"/>
       <c r="C52" s="12"/>
@@ -3941,10 +3833,8 @@
       <c r="AJ52" s="11"/>
       <c r="AK52" s="11"/>
       <c r="AL52" s="11"/>
-      <c r="AM52" s="11"/>
-      <c r="AN52" s="11"/>
-    </row>
-    <row r="53" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A53" s="11"/>
       <c r="B53" s="11"/>
       <c r="C53" s="12"/>
@@ -3983,10 +3873,8 @@
       <c r="AJ53" s="11"/>
       <c r="AK53" s="11"/>
       <c r="AL53" s="11"/>
-      <c r="AM53" s="11"/>
-      <c r="AN53" s="11"/>
-    </row>
-    <row r="54" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
       <c r="B54" s="11"/>
       <c r="C54" s="12"/>
@@ -4025,10 +3913,8 @@
       <c r="AJ54" s="11"/>
       <c r="AK54" s="11"/>
       <c r="AL54" s="11"/>
-      <c r="AM54" s="11"/>
-      <c r="AN54" s="11"/>
-    </row>
-    <row r="55" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A55" s="11"/>
       <c r="B55" s="11"/>
       <c r="C55" s="12"/>
@@ -4067,10 +3953,8 @@
       <c r="AJ55" s="11"/>
       <c r="AK55" s="11"/>
       <c r="AL55" s="11"/>
-      <c r="AM55" s="11"/>
-      <c r="AN55" s="11"/>
-    </row>
-    <row r="56" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A56" s="11"/>
       <c r="B56" s="11"/>
       <c r="C56" s="12"/>
@@ -4109,10 +3993,8 @@
       <c r="AJ56" s="11"/>
       <c r="AK56" s="11"/>
       <c r="AL56" s="11"/>
-      <c r="AM56" s="11"/>
-      <c r="AN56" s="11"/>
-    </row>
-    <row r="57" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A57" s="11"/>
       <c r="B57" s="11"/>
       <c r="C57" s="12"/>
@@ -4151,10 +4033,8 @@
       <c r="AJ57" s="11"/>
       <c r="AK57" s="11"/>
       <c r="AL57" s="11"/>
-      <c r="AM57" s="11"/>
-      <c r="AN57" s="11"/>
-    </row>
-    <row r="58" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A58" s="11"/>
       <c r="B58" s="11"/>
       <c r="C58" s="12"/>
@@ -4193,10 +4073,8 @@
       <c r="AJ58" s="11"/>
       <c r="AK58" s="11"/>
       <c r="AL58" s="11"/>
-      <c r="AM58" s="11"/>
-      <c r="AN58" s="11"/>
-    </row>
-    <row r="59" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A59" s="11"/>
       <c r="B59" s="11"/>
       <c r="C59" s="12"/>
@@ -4235,10 +4113,8 @@
       <c r="AJ59" s="11"/>
       <c r="AK59" s="11"/>
       <c r="AL59" s="11"/>
-      <c r="AM59" s="11"/>
-      <c r="AN59" s="11"/>
-    </row>
-    <row r="60" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A60" s="11"/>
       <c r="B60" s="11"/>
       <c r="C60" s="12"/>
@@ -4277,10 +4153,8 @@
       <c r="AJ60" s="11"/>
       <c r="AK60" s="11"/>
       <c r="AL60" s="11"/>
-      <c r="AM60" s="11"/>
-      <c r="AN60" s="11"/>
-    </row>
-    <row r="61" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A61" s="11"/>
       <c r="B61" s="11"/>
       <c r="C61" s="12"/>
@@ -4319,10 +4193,8 @@
       <c r="AJ61" s="11"/>
       <c r="AK61" s="11"/>
       <c r="AL61" s="11"/>
-      <c r="AM61" s="11"/>
-      <c r="AN61" s="11"/>
-    </row>
-    <row r="62" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A62" s="11"/>
       <c r="B62" s="11"/>
       <c r="C62" s="12"/>
@@ -4361,10 +4233,8 @@
       <c r="AJ62" s="11"/>
       <c r="AK62" s="11"/>
       <c r="AL62" s="11"/>
-      <c r="AM62" s="11"/>
-      <c r="AN62" s="11"/>
-    </row>
-    <row r="63" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A63" s="11"/>
       <c r="B63" s="11"/>
       <c r="C63" s="12"/>
@@ -4403,10 +4273,8 @@
       <c r="AJ63" s="11"/>
       <c r="AK63" s="11"/>
       <c r="AL63" s="11"/>
-      <c r="AM63" s="11"/>
-      <c r="AN63" s="11"/>
-    </row>
-    <row r="64" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A64" s="11"/>
       <c r="B64" s="11"/>
       <c r="C64" s="12"/>
@@ -4445,10 +4313,8 @@
       <c r="AJ64" s="11"/>
       <c r="AK64" s="11"/>
       <c r="AL64" s="11"/>
-      <c r="AM64" s="11"/>
-      <c r="AN64" s="11"/>
-    </row>
-    <row r="65" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A65" s="11"/>
       <c r="B65" s="11"/>
       <c r="C65" s="12"/>
@@ -4487,10 +4353,8 @@
       <c r="AJ65" s="11"/>
       <c r="AK65" s="11"/>
       <c r="AL65" s="11"/>
-      <c r="AM65" s="11"/>
-      <c r="AN65" s="11"/>
-    </row>
-    <row r="66" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A66" s="11"/>
       <c r="B66" s="11"/>
       <c r="C66" s="13"/>
@@ -4529,10 +4393,8 @@
       <c r="AJ66" s="11"/>
       <c r="AK66" s="11"/>
       <c r="AL66" s="11"/>
-      <c r="AM66" s="11"/>
-      <c r="AN66" s="11"/>
-    </row>
-    <row r="67" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A67" s="11"/>
       <c r="B67" s="11"/>
       <c r="C67" s="13"/>
@@ -4571,10 +4433,8 @@
       <c r="AJ67" s="11"/>
       <c r="AK67" s="11"/>
       <c r="AL67" s="11"/>
-      <c r="AM67" s="11"/>
-      <c r="AN67" s="11"/>
-    </row>
-    <row r="68" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A68" s="11"/>
       <c r="B68" s="11"/>
       <c r="C68" s="13"/>
@@ -4613,10 +4473,8 @@
       <c r="AJ68" s="11"/>
       <c r="AK68" s="11"/>
       <c r="AL68" s="11"/>
-      <c r="AM68" s="11"/>
-      <c r="AN68" s="11"/>
-    </row>
-    <row r="69" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A69" s="11"/>
       <c r="B69" s="11"/>
       <c r="C69" s="13"/>
@@ -4655,10 +4513,8 @@
       <c r="AJ69" s="11"/>
       <c r="AK69" s="11"/>
       <c r="AL69" s="11"/>
-      <c r="AM69" s="11"/>
-      <c r="AN69" s="11"/>
-    </row>
-    <row r="70" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A70" s="11"/>
       <c r="B70" s="11"/>
       <c r="C70" s="13"/>
@@ -4697,10 +4553,8 @@
       <c r="AJ70" s="11"/>
       <c r="AK70" s="11"/>
       <c r="AL70" s="11"/>
-      <c r="AM70" s="11"/>
-      <c r="AN70" s="11"/>
-    </row>
-    <row r="71" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A71" s="11"/>
       <c r="B71" s="11"/>
       <c r="C71" s="13"/>
@@ -4739,10 +4593,8 @@
       <c r="AJ71" s="11"/>
       <c r="AK71" s="11"/>
       <c r="AL71" s="11"/>
-      <c r="AM71" s="11"/>
-      <c r="AN71" s="11"/>
-    </row>
-    <row r="72" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A72" s="11"/>
       <c r="B72" s="11"/>
       <c r="C72" s="13"/>
@@ -4781,10 +4633,8 @@
       <c r="AJ72" s="11"/>
       <c r="AK72" s="11"/>
       <c r="AL72" s="11"/>
-      <c r="AM72" s="11"/>
-      <c r="AN72" s="11"/>
-    </row>
-    <row r="73" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A73" s="11"/>
       <c r="B73" s="11"/>
       <c r="C73" s="13"/>
@@ -4823,10 +4673,8 @@
       <c r="AJ73" s="11"/>
       <c r="AK73" s="11"/>
       <c r="AL73" s="11"/>
-      <c r="AM73" s="11"/>
-      <c r="AN73" s="11"/>
-    </row>
-    <row r="74" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A74" s="11"/>
       <c r="B74" s="11"/>
       <c r="C74" s="13"/>
@@ -4865,10 +4713,8 @@
       <c r="AJ74" s="11"/>
       <c r="AK74" s="11"/>
       <c r="AL74" s="11"/>
-      <c r="AM74" s="11"/>
-      <c r="AN74" s="11"/>
-    </row>
-    <row r="75" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A75" s="11"/>
       <c r="B75" s="11"/>
       <c r="C75" s="13"/>
@@ -4907,10 +4753,8 @@
       <c r="AJ75" s="11"/>
       <c r="AK75" s="11"/>
       <c r="AL75" s="11"/>
-      <c r="AM75" s="11"/>
-      <c r="AN75" s="11"/>
-    </row>
-    <row r="76" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A76" s="11"/>
       <c r="B76" s="11"/>
       <c r="C76" s="13"/>
@@ -4949,10 +4793,8 @@
       <c r="AJ76" s="11"/>
       <c r="AK76" s="11"/>
       <c r="AL76" s="11"/>
-      <c r="AM76" s="11"/>
-      <c r="AN76" s="11"/>
-    </row>
-    <row r="77" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A77" s="11"/>
       <c r="B77" s="11"/>
       <c r="C77" s="13"/>
@@ -4991,10 +4833,8 @@
       <c r="AJ77" s="11"/>
       <c r="AK77" s="11"/>
       <c r="AL77" s="11"/>
-      <c r="AM77" s="11"/>
-      <c r="AN77" s="11"/>
-    </row>
-    <row r="78" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A78" s="11"/>
       <c r="B78" s="11"/>
       <c r="C78" s="13"/>
@@ -5033,10 +4873,8 @@
       <c r="AJ78" s="11"/>
       <c r="AK78" s="11"/>
       <c r="AL78" s="11"/>
-      <c r="AM78" s="11"/>
-      <c r="AN78" s="11"/>
-    </row>
-    <row r="79" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A79" s="11"/>
       <c r="B79" s="11"/>
       <c r="C79" s="13"/>
@@ -5075,10 +4913,8 @@
       <c r="AJ79" s="11"/>
       <c r="AK79" s="11"/>
       <c r="AL79" s="11"/>
-      <c r="AM79" s="11"/>
-      <c r="AN79" s="11"/>
-    </row>
-    <row r="80" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A80" s="11"/>
       <c r="B80" s="11"/>
       <c r="C80" s="13"/>
@@ -5117,10 +4953,8 @@
       <c r="AJ80" s="11"/>
       <c r="AK80" s="11"/>
       <c r="AL80" s="11"/>
-      <c r="AM80" s="11"/>
-      <c r="AN80" s="11"/>
-    </row>
-    <row r="81" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A81" s="11"/>
       <c r="B81" s="11"/>
       <c r="C81" s="13"/>
@@ -5159,10 +4993,8 @@
       <c r="AJ81" s="11"/>
       <c r="AK81" s="11"/>
       <c r="AL81" s="11"/>
-      <c r="AM81" s="11"/>
-      <c r="AN81" s="11"/>
-    </row>
-    <row r="82" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A82" s="11"/>
       <c r="B82" s="11"/>
       <c r="C82" s="13"/>
@@ -5201,10 +5033,8 @@
       <c r="AJ82" s="11"/>
       <c r="AK82" s="11"/>
       <c r="AL82" s="11"/>
-      <c r="AM82" s="11"/>
-      <c r="AN82" s="11"/>
-    </row>
-    <row r="83" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A83" s="11"/>
       <c r="B83" s="11"/>
       <c r="C83" s="13"/>
@@ -5243,10 +5073,8 @@
       <c r="AJ83" s="11"/>
       <c r="AK83" s="11"/>
       <c r="AL83" s="11"/>
-      <c r="AM83" s="11"/>
-      <c r="AN83" s="11"/>
-    </row>
-    <row r="84" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="84" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A84" s="11"/>
       <c r="B84" s="11"/>
       <c r="C84" s="13"/>
@@ -5285,10 +5113,8 @@
       <c r="AJ84" s="11"/>
       <c r="AK84" s="11"/>
       <c r="AL84" s="11"/>
-      <c r="AM84" s="11"/>
-      <c r="AN84" s="11"/>
-    </row>
-    <row r="85" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A85" s="11"/>
       <c r="B85" s="11"/>
       <c r="C85" s="13"/>
@@ -5327,10 +5153,8 @@
       <c r="AJ85" s="11"/>
       <c r="AK85" s="11"/>
       <c r="AL85" s="11"/>
-      <c r="AM85" s="11"/>
-      <c r="AN85" s="11"/>
-    </row>
-    <row r="86" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A86" s="11"/>
       <c r="B86" s="11"/>
       <c r="C86" s="13"/>
@@ -5369,10 +5193,8 @@
       <c r="AJ86" s="11"/>
       <c r="AK86" s="11"/>
       <c r="AL86" s="11"/>
-      <c r="AM86" s="11"/>
-      <c r="AN86" s="11"/>
-    </row>
-    <row r="87" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A87" s="11"/>
       <c r="B87" s="11"/>
       <c r="C87" s="13"/>
@@ -5411,10 +5233,8 @@
       <c r="AJ87" s="11"/>
       <c r="AK87" s="11"/>
       <c r="AL87" s="11"/>
-      <c r="AM87" s="11"/>
-      <c r="AN87" s="11"/>
-    </row>
-    <row r="88" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A88" s="11"/>
       <c r="B88" s="11"/>
       <c r="C88" s="13"/>
@@ -5453,10 +5273,8 @@
       <c r="AJ88" s="11"/>
       <c r="AK88" s="11"/>
       <c r="AL88" s="11"/>
-      <c r="AM88" s="11"/>
-      <c r="AN88" s="11"/>
-    </row>
-    <row r="89" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A89" s="11"/>
       <c r="B89" s="11"/>
       <c r="C89" s="13"/>
@@ -5495,10 +5313,8 @@
       <c r="AJ89" s="11"/>
       <c r="AK89" s="11"/>
       <c r="AL89" s="11"/>
-      <c r="AM89" s="11"/>
-      <c r="AN89" s="11"/>
-    </row>
-    <row r="90" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A90" s="11"/>
       <c r="B90" s="11"/>
       <c r="C90" s="13"/>
@@ -5537,10 +5353,8 @@
       <c r="AJ90" s="11"/>
       <c r="AK90" s="11"/>
       <c r="AL90" s="11"/>
-      <c r="AM90" s="11"/>
-      <c r="AN90" s="11"/>
-    </row>
-    <row r="91" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A91" s="11"/>
       <c r="B91" s="11"/>
       <c r="C91" s="13"/>
@@ -5579,10 +5393,8 @@
       <c r="AJ91" s="11"/>
       <c r="AK91" s="11"/>
       <c r="AL91" s="11"/>
-      <c r="AM91" s="11"/>
-      <c r="AN91" s="11"/>
-    </row>
-    <row r="92" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A92" s="11"/>
       <c r="B92" s="11"/>
       <c r="C92" s="13"/>
@@ -5621,10 +5433,8 @@
       <c r="AJ92" s="11"/>
       <c r="AK92" s="11"/>
       <c r="AL92" s="11"/>
-      <c r="AM92" s="11"/>
-      <c r="AN92" s="11"/>
-    </row>
-    <row r="93" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="93" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A93" s="11"/>
       <c r="B93" s="11"/>
       <c r="C93" s="13"/>
@@ -5663,10 +5473,8 @@
       <c r="AJ93" s="11"/>
       <c r="AK93" s="11"/>
       <c r="AL93" s="11"/>
-      <c r="AM93" s="11"/>
-      <c r="AN93" s="11"/>
-    </row>
-    <row r="94" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A94" s="11"/>
       <c r="B94" s="11"/>
       <c r="C94" s="13"/>
@@ -5705,10 +5513,8 @@
       <c r="AJ94" s="11"/>
       <c r="AK94" s="11"/>
       <c r="AL94" s="11"/>
-      <c r="AM94" s="11"/>
-      <c r="AN94" s="11"/>
-    </row>
-    <row r="95" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="95" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A95" s="11"/>
       <c r="B95" s="11"/>
       <c r="C95" s="13"/>
@@ -5747,10 +5553,8 @@
       <c r="AJ95" s="11"/>
       <c r="AK95" s="11"/>
       <c r="AL95" s="11"/>
-      <c r="AM95" s="11"/>
-      <c r="AN95" s="11"/>
-    </row>
-    <row r="96" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A96" s="11"/>
       <c r="B96" s="11"/>
       <c r="C96" s="13"/>
@@ -5789,10 +5593,8 @@
       <c r="AJ96" s="11"/>
       <c r="AK96" s="11"/>
       <c r="AL96" s="11"/>
-      <c r="AM96" s="11"/>
-      <c r="AN96" s="11"/>
-    </row>
-    <row r="97" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="97" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A97" s="11"/>
       <c r="B97" s="11"/>
       <c r="C97" s="13"/>
@@ -5831,10 +5633,8 @@
       <c r="AJ97" s="11"/>
       <c r="AK97" s="11"/>
       <c r="AL97" s="11"/>
-      <c r="AM97" s="11"/>
-      <c r="AN97" s="11"/>
-    </row>
-    <row r="98" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A98" s="11"/>
       <c r="B98" s="11"/>
       <c r="C98" s="13"/>
@@ -5873,10 +5673,8 @@
       <c r="AJ98" s="11"/>
       <c r="AK98" s="11"/>
       <c r="AL98" s="11"/>
-      <c r="AM98" s="11"/>
-      <c r="AN98" s="11"/>
-    </row>
-    <row r="99" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="99" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A99" s="11"/>
       <c r="B99" s="11"/>
       <c r="C99" s="13"/>
@@ -5915,10 +5713,8 @@
       <c r="AJ99" s="11"/>
       <c r="AK99" s="11"/>
       <c r="AL99" s="11"/>
-      <c r="AM99" s="11"/>
-      <c r="AN99" s="11"/>
-    </row>
-    <row r="100" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="100" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A100" s="11"/>
       <c r="B100" s="11"/>
       <c r="C100" s="13"/>
@@ -5957,10 +5753,8 @@
       <c r="AJ100" s="11"/>
       <c r="AK100" s="11"/>
       <c r="AL100" s="11"/>
-      <c r="AM100" s="11"/>
-      <c r="AN100" s="11"/>
-    </row>
-    <row r="101" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A101" s="11"/>
       <c r="B101" s="11"/>
       <c r="C101" s="13"/>
@@ -5999,10 +5793,8 @@
       <c r="AJ101" s="11"/>
       <c r="AK101" s="11"/>
       <c r="AL101" s="11"/>
-      <c r="AM101" s="11"/>
-      <c r="AN101" s="11"/>
-    </row>
-    <row r="102" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="102" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A102" s="11"/>
       <c r="B102" s="11"/>
       <c r="C102" s="13"/>
@@ -6041,10 +5833,8 @@
       <c r="AJ102" s="11"/>
       <c r="AK102" s="11"/>
       <c r="AL102" s="11"/>
-      <c r="AM102" s="11"/>
-      <c r="AN102" s="11"/>
-    </row>
-    <row r="103" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A103" s="11"/>
       <c r="B103" s="11"/>
       <c r="C103" s="13"/>
@@ -6083,10 +5873,8 @@
       <c r="AJ103" s="11"/>
       <c r="AK103" s="11"/>
       <c r="AL103" s="11"/>
-      <c r="AM103" s="11"/>
-      <c r="AN103" s="11"/>
-    </row>
-    <row r="104" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="104" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A104" s="11"/>
       <c r="B104" s="11"/>
       <c r="C104" s="13"/>
@@ -6125,10 +5913,8 @@
       <c r="AJ104" s="11"/>
       <c r="AK104" s="11"/>
       <c r="AL104" s="11"/>
-      <c r="AM104" s="11"/>
-      <c r="AN104" s="11"/>
-    </row>
-    <row r="105" spans="1:40" x14ac:dyDescent="0.25">
+    </row>
+    <row r="105" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A105" s="11"/>
       <c r="B105" s="11"/>
       <c r="C105" s="13"/>
@@ -6167,8 +5953,6 @@
       <c r="AJ105" s="11"/>
       <c r="AK105" s="11"/>
       <c r="AL105" s="11"/>
-      <c r="AM105" s="11"/>
-      <c r="AN105" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>